<commit_message>
Complete mobile checks and simplify documentation
</commit_message>
<xml_diff>
--- a/lab02/bugs.xlsx
+++ b/lab02/bugs.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Дефекты" sheetId="1" r:id="R9aeb61bb49c74f0d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Описание" sheetId="2" r:id="Rde5357117e574620"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Дефекты" sheetId="1" r:id="R51b2971932214f22"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Описание" sheetId="2" r:id="Rc9a361c2a4774933"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -569,7 +569,7 @@
     </x:row>
     <x:row r="13" ht="42" customHeight="1">
       <x:c r="A13" s="9" t="str">
-        <x:v>Время прогона</x:v>
+        <x:v>Время прогона (UTC)</x:v>
       </x:c>
       <x:c r="B13" s="12" t="d">
         <x:v>2026-10-27T23:03:24.007Z</x:v>
@@ -657,7 +657,7 @@
     </x:row>
     <x:row r="25" ht="42" customHeight="1">
       <x:c r="A25" s="9" t="str">
-        <x:v>Время прогона</x:v>
+        <x:v>Время прогона (UTC)</x:v>
       </x:c>
       <x:c r="B25" s="12" t="d">
         <x:v>2026-10-27T23:03:24.007Z</x:v>
@@ -745,7 +745,7 @@
     </x:row>
     <x:row r="37" ht="42" customHeight="1">
       <x:c r="A37" s="9" t="str">
-        <x:v>Время прогона</x:v>
+        <x:v>Время прогона (UTC)</x:v>
       </x:c>
       <x:c r="B37" s="12" t="d">
         <x:v>2026-10-27T23:03:24.007Z</x:v>
@@ -833,7 +833,7 @@
     </x:row>
     <x:row r="49" ht="42" customHeight="1">
       <x:c r="A49" s="9" t="str">
-        <x:v>Время прогона</x:v>
+        <x:v>Время прогона (UTC)</x:v>
       </x:c>
       <x:c r="B49" s="12" t="d">
         <x:v>2026-10-27T23:03:24.007Z</x:v>

</xml_diff>